<commit_message>
Data wrangling - new data integration from 2024-2025
After being handed over the main database with data from 2020-24, we received a new extraction from a posterior period, including patient data from 2024-25. This must be added to the existing databases.

To do that, created a new cell under Import raw files once paths are defined / Add new data entries to existing 'raw' database.

This functionality accesses the defined new extraction, checks if the table structures match the existing database tables, and whether the new data is indeed new, and if both checks pass, new data is integrated into the database. If they fail, manual adjustments or revisions are needed on the new data.

Entered 2024-25 data from over 1500 new patients - but only 2 patients passed the eventual research-ready filtration, because apparently, they did not consent to the research use of their data!
</commit_message>
<xml_diff>
--- a/DB2_26Feb26_intact/pac.xlsx
+++ b/DB2_26Feb26_intact/pac.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://proteinsolution-my.sharepoint.com/personal/drobles_pronokal_com/Documents/Escritorio/v4 2024_03_2025/entregable/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="75" documentId="8_{DF0EAC5F-AF94-4837-9F56-03A6D3088AAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E53B4401-003A-47EE-AFE7-E9375D478851}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4506"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19420" windowHeight="11020"/>
   </bookViews>
   <sheets>
     <sheet name="pac_cientifico" sheetId="1" r:id="rId1"/>
@@ -4998,7 +4992,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -5033,12 +5027,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normál" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -5050,6 +5041,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -5065,22 +5059,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M1626" totalsRowShown="0">
-  <autoFilter ref="A1:M1626" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:M1626" totalsRowShown="0">
+  <autoFilter ref="A1:M1626"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{7C224378-8F5F-47CF-92DE-873FF09EC01D}" name="Id Paciente" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Fecha de creación"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Sexo" dataDxfId="4"/>
-    <tableColumn id="18" xr3:uid="{5673CF71-155F-460F-ABC0-7DFEE8B9A0F6}" name="Compra Online" dataDxfId="3"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Patient Collective"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="NAV Company Lower"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Fecha de nacimiento"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="GDPR-4"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Fecha GDPR-4"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="GDPR-10"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Fecha GDPR-10"/>
-    <tableColumn id="2" xr3:uid="{2E5E3CFE-BE01-4091-8729-9E6F3C10FB27}" name="genomics_available" dataDxfId="2"/>
-    <tableColumn id="19" xr3:uid="{0CE2C0B1-8005-49C2-8AB8-87B485ACA289}" name="Muestra" dataDxfId="1"/>
+    <tableColumn id="1" name="Id Paciente" dataDxfId="4"/>
+    <tableColumn id="5" name="Fecha de creación"/>
+    <tableColumn id="6" name="Sexo" dataDxfId="3"/>
+    <tableColumn id="18" name="Compra Online" dataDxfId="2"/>
+    <tableColumn id="8" name="Patient Collective"/>
+    <tableColumn id="9" name="NAV Company Lower"/>
+    <tableColumn id="10" name="Fecha de nacimiento"/>
+    <tableColumn id="13" name="GDPR-4"/>
+    <tableColumn id="14" name="Fecha GDPR-4"/>
+    <tableColumn id="15" name="GDPR-10"/>
+    <tableColumn id="16" name="Fecha GDPR-10"/>
+    <tableColumn id="2" name="genomics_available" dataDxfId="1"/>
+    <tableColumn id="19" name="Muestra" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5129,7 +5123,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -5181,7 +5175,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -5395,17 +5389,17 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="dataSheet"/>
   <dimension ref="A1:M1626"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="28" style="4" customWidth="1"/>
     <col min="2" max="2" width="28" style="2" customWidth="1"/>
@@ -52681,20 +52675,20 @@
     </row>
   </sheetData>
   <dataValidations count="6">
-    <dataValidation allowBlank="1" errorTitle="Valor de lista" error="Compra Genomics debe estar seleccionado en la lista desplegable." promptTitle="Conjunto de opciones" prompt="Seleccione un valor de la lista desplegable." sqref="L2:M1626" xr:uid="{25BB0301-C2F0-48FA-9AD3-5B611B3F96D0}"/>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Fecha de creación debe estar en el formato de fecha y hora correcto." promptTitle="Fecha y hora" prompt=" " sqref="B2:C1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation allowBlank="1" errorTitle="Valor de lista" error="Compra Genomics debe estar seleccionado en la lista desplegable." promptTitle="Conjunto de opciones" prompt="Seleccione un valor de la lista desplegable." sqref="L2:M1626"/>
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Fecha de creación debe estar en el formato de fecha y hora correcto." promptTitle="Fecha y hora" prompt=" " sqref="B2:C1048576">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Longitud excedida" error="Este valor debe tener 4000 caracteres o menos." promptTitle="Texto" prompt="Longitud máxima: 4000 caracteres." sqref="G1627:G1048576 F2:F1626" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="textLength" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Longitud excedida" error="Este valor debe tener 4000 caracteres o menos." promptTitle="Texto" prompt="Longitud máxima: 4000 caracteres." sqref="G1627:G1048576 F2:F1626">
       <formula1>4000</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Fecha de nacimiento debe estar en el formato de fecha correcto." promptTitle="Fecha" prompt=" " sqref="G2:G1626" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Fecha de nacimiento debe estar en el formato de fecha correcto." promptTitle="Fecha" prompt=" " sqref="G2:G1626">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Fecha autorización uso datos estudios médicos debe estar en el formato de fecha y hora correcto." promptTitle="Fecha y hora" prompt=" " sqref="J1627:J1048576 I2:I1626" xr:uid="{00000000-0002-0000-0000-00000B000000}">
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Fecha autorización uso datos estudios médicos debe estar en el formato de fecha y hora correcto." promptTitle="Fecha y hora" prompt=" " sqref="J1627:J1048576 I2:I1626">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Fecha autorización datos de salud y genéticos debe estar en el formato de fecha y hora correcto." promptTitle="Fecha y hora" prompt=" " sqref="L1627:L1048576 K2:K1626" xr:uid="{00000000-0002-0000-0000-00000D000000}">
+    <dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Fecha autorización datos de salud y genéticos debe estar en el formato de fecha y hora correcto." promptTitle="Fecha y hora" prompt=" " sqref="L1627:L1048576 K2:K1626">
       <formula1>1</formula1>
     </dataValidation>
   </dataValidations>
@@ -52702,7 +52696,7 @@
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
-  <extLst>
+  <extLst xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor de lista" error="Compra Genomics debe estar seleccionado en la lista desplegable." promptTitle="Conjunto de opciones" prompt="Seleccione un valor de la lista desplegable." xr:uid="{00000000-0002-0000-0000-00000E000000}">
@@ -52754,10 +52748,10 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="hiddenDataSheet"/>
   <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">

</xml_diff>